<commit_message>
data: sync PC-server-0148 2026-09-24 10:54
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N544"/>
+  <dimension ref="A1:N551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29850,6 +29850,368 @@
         <v>0</v>
       </c>
     </row>
+    <row r="545">
+      <c r="A545" t="n">
+        <v>1296534</v>
+      </c>
+      <c r="B545" t="n">
+        <v>1</v>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>2026-09-24 06:43:06</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:43:06</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr"/>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:43:06</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr"/>
+      <c r="M545" t="inlineStr"/>
+      <c r="N545" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="n">
+        <v>1296478</v>
+      </c>
+      <c r="B546" t="n">
+        <v>1</v>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr"/>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>2026-09-24 02:52:35</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:12:35</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr"/>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:12:35</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr"/>
+      <c r="M546" t="inlineStr"/>
+      <c r="N546" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="n">
+        <v>1296471</v>
+      </c>
+      <c r="B547" t="n">
+        <v>1</v>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr"/>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>2026-09-24 02:47:39</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:07:39</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr"/>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:07:39</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr"/>
+      <c r="M547" t="inlineStr"/>
+      <c r="N547" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="n">
+        <v>1296583</v>
+      </c>
+      <c r="B548" t="n">
+        <v>0</v>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr"/>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>2026-09-24 08:55:34</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>2026-09-24 09:15:34</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>HO</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr"/>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>2026-09-24 09:15:34</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr"/>
+      <c r="M548" t="inlineStr"/>
+      <c r="N548" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="n">
+        <v>1296597</v>
+      </c>
+      <c r="B549" t="n">
+        <v>0</v>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>2026-09-24 09:10:04</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:10:04</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr"/>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:10:04</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr"/>
+      <c r="M549" t="inlineStr"/>
+      <c r="N549" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="n">
+        <v>1296583</v>
+      </c>
+      <c r="B550" t="n">
+        <v>1</v>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr"/>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>2026-09-24 08:55:34</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>2026-09-24 09:15:34</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>HO</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr"/>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>2026-09-24 09:15:34</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr"/>
+      <c r="M550" t="inlineStr"/>
+      <c r="N550" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="n">
+        <v>1296765</v>
+      </c>
+      <c r="B551" t="n">
+        <v>0</v>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>每日质量不达标</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:00:00</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>2026-09-25 10:00:00</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr"/>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>2026-09-25 10:00:00</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr"/>
+      <c r="M551" t="inlineStr"/>
+      <c r="N551" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-23 08:38
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N725"/>
+  <dimension ref="A1:N726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39324,6 +39324,56 @@
         <v>0</v>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="n">
+        <v>1323190</v>
+      </c>
+      <c r="B726" t="n">
+        <v>1</v>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr"/>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>2026-10-23 07:49:15</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>2026-10-23 08:09:15</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>9H</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr"/>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K726" t="inlineStr">
+        <is>
+          <t>2026-10-23 08:09:15</t>
+        </is>
+      </c>
+      <c r="L726" t="inlineStr"/>
+      <c r="M726" t="inlineStr"/>
+      <c r="N726" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-23 09:05
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N726"/>
+  <dimension ref="A1:N727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39374,6 +39374,60 @@
         <v>0</v>
       </c>
     </row>
+    <row r="727">
+      <c r="A727" t="n">
+        <v>1323218</v>
+      </c>
+      <c r="B727" t="n">
+        <v>0</v>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>2026-10-23 08:44:33</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>2026-10-23 09:44:33</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr"/>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K727" t="inlineStr">
+        <is>
+          <t>2026-10-23 09:44:33</t>
+        </is>
+      </c>
+      <c r="L727" t="inlineStr"/>
+      <c r="M727" t="inlineStr"/>
+      <c r="N727" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-23 09:11
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N727"/>
+  <dimension ref="A1:N733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39428,6 +39428,322 @@
         <v>0</v>
       </c>
     </row>
+    <row r="728">
+      <c r="A728" t="n">
+        <v>1323022</v>
+      </c>
+      <c r="B728" t="n">
+        <v>1</v>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr"/>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:28:20</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:48:20</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>9H</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr"/>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K728" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:48:20</t>
+        </is>
+      </c>
+      <c r="L728" t="inlineStr"/>
+      <c r="M728" t="inlineStr"/>
+      <c r="N728" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="n">
+        <v>1322931</v>
+      </c>
+      <c r="B729" t="n">
+        <v>1</v>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:52:14</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:52:14</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr"/>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K729" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:52:14</t>
+        </is>
+      </c>
+      <c r="L729" t="inlineStr"/>
+      <c r="M729" t="inlineStr"/>
+      <c r="N729" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="n">
+        <v>1322910</v>
+      </c>
+      <c r="B730" t="n">
+        <v>1</v>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr"/>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:40:29</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:00:29</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>9H</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr"/>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K730" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:00:29</t>
+        </is>
+      </c>
+      <c r="L730" t="inlineStr"/>
+      <c r="M730" t="inlineStr"/>
+      <c r="N730" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="n">
+        <v>1322861</v>
+      </c>
+      <c r="B731" t="n">
+        <v>1</v>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:45:58</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:45:58</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr"/>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K731" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:45:58</t>
+        </is>
+      </c>
+      <c r="L731" t="inlineStr"/>
+      <c r="M731" t="inlineStr"/>
+      <c r="N731" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="n">
+        <v>1322679</v>
+      </c>
+      <c r="B732" t="n">
+        <v>1</v>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:11:28</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:11:28</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr"/>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K732" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:11:28</t>
+        </is>
+      </c>
+      <c r="L732" t="inlineStr"/>
+      <c r="M732" t="inlineStr"/>
+      <c r="N732" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="n">
+        <v>1322623</v>
+      </c>
+      <c r="B733" t="n">
+        <v>0</v>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>每日质量不达标</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:00:00</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>2026-10-23 10:00:00</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr"/>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K733" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:00:06</t>
+        </is>
+      </c>
+      <c r="L733" t="inlineStr"/>
+      <c r="M733" t="inlineStr"/>
+      <c r="N733" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-24 08:12
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N744"/>
+  <dimension ref="A1:N752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40326,6 +40326,426 @@
         <v>1</v>
       </c>
     </row>
+    <row r="745">
+      <c r="A745" t="n">
+        <v>1324163</v>
+      </c>
+      <c r="B745" t="n">
+        <v>1</v>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:50:59</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>2026-10-24 04:50:59</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr"/>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K745" t="inlineStr">
+        <is>
+          <t>2026-10-24 04:50:59</t>
+        </is>
+      </c>
+      <c r="L745" t="inlineStr"/>
+      <c r="M745" t="inlineStr"/>
+      <c r="N745" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="n">
+        <v>1324114</v>
+      </c>
+      <c r="B746" t="n">
+        <v>1</v>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:50:04</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:10:04</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>9H</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr"/>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K746" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:10:04</t>
+        </is>
+      </c>
+      <c r="L746" t="inlineStr"/>
+      <c r="M746" t="inlineStr"/>
+      <c r="N746" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="n">
+        <v>1324100</v>
+      </c>
+      <c r="B747" t="n">
+        <v>1</v>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:32:07</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:32:07</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr"/>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K747" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:32:07</t>
+        </is>
+      </c>
+      <c r="L747" t="inlineStr"/>
+      <c r="M747" t="inlineStr"/>
+      <c r="N747" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="n">
+        <v>1324086</v>
+      </c>
+      <c r="B748" t="n">
+        <v>1</v>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:31:24</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:31:24</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr"/>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>2026-10-23 22:31:24</t>
+        </is>
+      </c>
+      <c r="L748" t="inlineStr"/>
+      <c r="M748" t="inlineStr"/>
+      <c r="N748" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="n">
+        <v>1324058</v>
+      </c>
+      <c r="B749" t="n">
+        <v>1</v>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:03:49</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>2026-10-24 03:03:49</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr"/>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K749" t="inlineStr">
+        <is>
+          <t>2026-10-24 03:03:49</t>
+        </is>
+      </c>
+      <c r="L749" t="inlineStr"/>
+      <c r="M749" t="inlineStr"/>
+      <c r="N749" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="n">
+        <v>1324037</v>
+      </c>
+      <c r="B750" t="n">
+        <v>1</v>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>2026-10-23 20:42:53</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:02:53</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr"/>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K750" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:02:53</t>
+        </is>
+      </c>
+      <c r="L750" t="inlineStr"/>
+      <c r="M750" t="inlineStr"/>
+      <c r="N750" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>1324009</v>
+      </c>
+      <c r="B751" t="n">
+        <v>1</v>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:45:51</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>2026-10-23 20:00:51</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr"/>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K751" t="inlineStr">
+        <is>
+          <t>2026-10-23 20:00:51</t>
+        </is>
+      </c>
+      <c r="L751" t="inlineStr"/>
+      <c r="M751" t="inlineStr"/>
+      <c r="N751" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>1323862</v>
+      </c>
+      <c r="B752" t="n">
+        <v>1</v>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>2026-10-23 17:53:37</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>2026-10-23 18:13:37</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr"/>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K752" t="inlineStr">
+        <is>
+          <t>2026-10-23 18:13:37</t>
+        </is>
+      </c>
+      <c r="L752" t="inlineStr"/>
+      <c r="M752" t="inlineStr"/>
+      <c r="N752" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-26 08:19
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N752"/>
+  <dimension ref="A1:N754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40746,6 +40746,114 @@
         <v>0</v>
       </c>
     </row>
+    <row r="753">
+      <c r="A753" t="n">
+        <v>1325822</v>
+      </c>
+      <c r="B753" t="n">
+        <v>1</v>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>2026-10-26 03:55:34</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:55:34</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr"/>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K753" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:55:34</t>
+        </is>
+      </c>
+      <c r="L753" t="inlineStr"/>
+      <c r="M753" t="inlineStr"/>
+      <c r="N753" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>1325059</v>
+      </c>
+      <c r="B754" t="n">
+        <v>1</v>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>2026-10-25 04:03:50</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>2026-10-25 05:03:50</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr"/>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K754" t="inlineStr">
+        <is>
+          <t>2026-10-25 05:03:50</t>
+        </is>
+      </c>
+      <c r="L754" t="inlineStr"/>
+      <c r="M754" t="inlineStr"/>
+      <c r="N754" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: sync PC-server-0148 2026-10-27 08:21
</commit_message>
<xml_diff>
--- a/data/携程.xlsx
+++ b/data/携程.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N754"/>
+  <dimension ref="A1:N755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40854,6 +40854,60 @@
         <v>0</v>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>1326312</v>
+      </c>
+      <c r="B755" t="n">
+        <v>1</v>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>NDC质量不达标禁售</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>实时质量不达标</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57:12</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>2026-10-26 23:57:12</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr"/>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="K755" t="inlineStr">
+        <is>
+          <t>2026-10-26 23:57:12</t>
+        </is>
+      </c>
+      <c r="L755" t="inlineStr"/>
+      <c r="M755" t="inlineStr"/>
+      <c r="N755" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>